<commit_message>
Update summary with container/transport reference (MBL received)
- Container OOCU9736647 / seal 40305210 / 40HC
- Master B/L GMNNPRG260600050 (Globelink); on-board 25/06/2026, telex released
- Measurement revised to 19.940 m3; destination agent Austromar (EORI CZ6047184)
- Flag routing discrepancy: HBL discharge Hamburg vs MBL discharge Prague
- Goods data (INV/PL) unchanged; still no preferencni veta

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDi54333RkSSDjzgisDWnP
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_HPE_1374217.xlsx
+++ b/output/HS_Code_Summary_HPE_1374217.xlsx
@@ -103,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,6 +134,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -723,20 +724,75 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>Transport / container reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>• Container No.: OOCU9736647  |  Seal: 40305210  |  Type: 40HC (40ft high-cube).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>• Master B/L: GMNNPRG260600050 (Globelink Container Lines)  |  House B/L: XH26060361 (Star Ocean Logistics).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>• On-board date: 25/06/2026 (vessel DANUM 175, voy. 117S; loaded Manila). Telex released / Express B/L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>• Measurement revised to 19.940 m3 (was 19.239); gross incl. pallets 2,750.20 kg unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>• Destination customs agent / declarant: Austromar obchodni a dopravni spol. s r.o., Praha (EORI CZ6047184).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>⚠ Routing discrepancy: House B/L shows discharge HAMBURG -&gt; Kutna Hora; Master B/L shows discharge PRAGUE. Confirm actual clearance point with the forwarder.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A11:I11"/>
+  <mergeCells count="19">
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A21:I21"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A13:I13"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A12:I12"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A11:I11"/>
     <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>